<commit_message>
deploy: main → 7a181a25b9be1415ba6c91ef2d335ce5f077a36a
</commit_message>
<xml_diff>
--- a/StructureDefinition-SEEHDSAuditEventReadAccessLog.xlsx
+++ b/StructureDefinition-SEEHDSAuditEventReadAccessLog.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-07T11:49:57+00:00</t>
+    <t>2026-10-09T07:52:45+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -488,7 +488,7 @@
 </t>
   </si>
   <si>
-    <t>Händelsetyp (accessType)</t>
+    <t>Händelsetyp – fast värde, meddelandet saknar åtkomsttyp (LOG-002)</t>
   </si>
   <si>
     <t>Identifier for a family of the event.  For example, a menu item, program, rule, policy, function code, application name or URL. It identifies the performed function.</t>
@@ -524,7 +524,7 @@
     <t>AuditEvent.subtype</t>
   </si>
   <si>
-    <t>Händelseundertyp (accessSubType)</t>
+    <t>More specific type/id for the event</t>
   </si>
   <si>
     <t>Identifier for the category of event.</t>
@@ -607,7 +607,7 @@
 </t>
   </si>
   <si>
-    <t>Loggtidpunkt (accessTime)</t>
+    <t>Tidpunkt för åtkomst (accessLog.accessDate)</t>
   </si>
   <si>
     <t>The time when the event was recorded.</t>
@@ -634,7 +634,7 @@
     <t>AuditEvent.outcome</t>
   </si>
   <si>
-    <t>Utfall (accessOutcome)</t>
+    <t>Utfall – 0 (Success): loggposten avser en genomförd åtkomst</t>
   </si>
   <si>
     <t>Indicates whether the event succeeded or failed.</t>
@@ -862,11 +862,11 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(https://fhir.inera.se/ig/ehds-tk/StructureDefinition/SEEHDSPractitionerRole|Device)
+    <t xml:space="preserve">Reference(https://fhir.inera.se/ig/ehds-tk/StructureDefinition/SEEHDSPractitionerRole|https://fhir.inera.se/ig/ehds-tk/StructureDefinition/SEEHDSOrganization|Device)
 </t>
   </si>
   <si>
-    <t>Användare/system (userId)</t>
+    <t>Användare (accessLog.userId), vårdenhet (careUnitId) eller vårdgivare (careProviderId)</t>
   </si>
   <si>
     <t>Reference to who this agent is that was involved in the event.</t>
@@ -1102,7 +1102,7 @@
     <t>AuditEvent.agent.purposeOfUse</t>
   </si>
   <si>
-    <t>Åtkomstsyfte (accessPurpose)</t>
+    <t>Åtkomstsyfte (accessLog.purpose)</t>
   </si>
   <si>
     <t>The reason (purpose of use), specific to this agent, that was used during the event being recorded.</t>
@@ -1181,7 +1181,7 @@
 </t>
   </si>
   <si>
-    <t>Loggkälla/system (sourceSystemHSAId)</t>
+    <t>Det källsystem (logisk adress) som bryggan anropade</t>
   </si>
   <si>
     <t>Identifier of the source where the event was detected.</t>
@@ -1268,7 +1268,7 @@
 </t>
   </si>
   <si>
-    <t>Patientidentifierare (patientId)</t>
+    <t>Patient – den efterfrågade patienten (begärans patientId)</t>
   </si>
   <si>
     <t>Identifies a specific instance of the entity. The reference should be version specific.</t>
@@ -1856,7 +1856,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="93.98828125" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="130.84375" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -3217,7 +3217,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" hidden="true">
       <c r="A12" t="s" s="2">
         <v>161</v>
       </c>
@@ -3236,7 +3236,7 @@
         <v>81</v>
       </c>
       <c r="H12" t="s" s="2">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="I12" t="s" s="2">
         <v>79</v>

</xml_diff>